<commit_message>
fix: move Oneng Sumarni to tidak_acc_layak_huni, remove duplicate ONENG entry
- Oneng Sumarni (entry 47) changed from data_acc to tidak_acc_layak_huni
- Keterangan: Diganti oleh Tomi Harun Arasyid
- Removed duplicate entry 56 (ONENG) since it's the same person
- Photos already exist at /dokumentasi/lampegan/oneng sumarni
- Lampegan: 15 data_acc, 7 diganti, 1 tidak melanjutkan
- Regenerated Excel, Word, PDF documents
</commit_message>
<xml_diff>
--- a/public/outputs/Data_BSPS_Paseh_Loa_Lampegan.xlsx
+++ b/public/outputs/Data_BSPS_Paseh_Loa_Lampegan.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3419,63 +3419,63 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>ONENG SUMARNI</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>3204364808810005</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>3204361903057024</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>Kp Lampegan</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr">
+      <c r="H48" s="5" t="inlineStr">
         <is>
           <t>Lampegan</t>
         </is>
       </c>
-      <c r="I48" s="3" t="inlineStr">
+      <c r="I48" s="5" t="inlineStr">
         <is>
           <t>Ibun</t>
         </is>
       </c>
-      <c r="J48" s="2" t="n">
+      <c r="J48" s="4" t="n">
         <v>-7.023</v>
       </c>
-      <c r="K48" s="2" t="n">
+      <c r="K48" s="4" t="n">
         <v>107.5655</v>
       </c>
-      <c r="L48" s="3" t="inlineStr">
-        <is>
-          <t>Data Acc</t>
-        </is>
-      </c>
-      <c r="M48" s="3" t="inlineStr">
-        <is>
-          <t>Backlog 2 Desil 3</t>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>Tidak Acc Layak Huni</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>Diganti oleh Tomi Harun Arasyid</t>
         </is>
       </c>
     </row>
@@ -3964,67 +3964,6 @@
       <c r="M56" s="5" t="inlineStr">
         <is>
           <t>Diganti oleh Cecep</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>ONENG</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>Kp Lampegan</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H57" s="5" t="inlineStr">
-        <is>
-          <t>Lampegan</t>
-        </is>
-      </c>
-      <c r="I57" s="5" t="inlineStr">
-        <is>
-          <t>Ibun</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="n">
-        <v>-7.0218</v>
-      </c>
-      <c r="K57" s="4" t="n">
-        <v>107.5642</v>
-      </c>
-      <c r="L57" s="5" t="inlineStr">
-        <is>
-          <t>Tidak Acc Layak Huni</t>
-        </is>
-      </c>
-      <c r="M57" s="5" t="inlineStr">
-        <is>
-          <t>Diganti oleh Tomi Harun Arasyid</t>
         </is>
       </c>
     </row>
@@ -4039,7 +3978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6143,32 +6082,32 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>ONENG SUMARNI</t>
+          <t>ENCAR</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>3204364808810005</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>3204361903057024</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Kp Lampegan</t>
+          <t>KP. Awilega RT 3 RW 9</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -6182,10 +6121,10 @@
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>-7.023</v>
+        <v>-7.026</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>107.5655</v>
+        <v>107.563</v>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
@@ -6194,7 +6133,7 @@
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>Backlog 2 Desil 3</t>
+          <t>Backlog 2 - Pengganti Wawan Setiawan</t>
         </is>
       </c>
     </row>
@@ -6204,32 +6143,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>ENCAR</t>
+          <t>TOMI HARUN ARASYID</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3204360505780007</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3204360906051418</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>KP. Awilega RT 3 RW 9</t>
+          <t>KP. Lampegan RT 003 RW 005</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>005</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -6243,10 +6182,10 @@
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>-7.026</v>
+        <v>-7.022</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>107.563</v>
+        <v>107.564</v>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
@@ -6254,67 +6193,6 @@
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
-        <is>
-          <t>Backlog 2 - Pengganti Wawan Setiawan</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>TOMI HARUN ARASYID</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>3204360505780007</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>3204360906051418</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>KP. Lampegan RT 003 RW 005</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>003</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>005</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>Lampegan</t>
-        </is>
-      </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>Ibun</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="n">
-        <v>-7.022</v>
-      </c>
-      <c r="K37" s="2" t="n">
-        <v>107.564</v>
-      </c>
-      <c r="L37" s="3" t="inlineStr">
-        <is>
-          <t>Data Acc</t>
-        </is>
-      </c>
-      <c r="M37" s="3" t="inlineStr">
         <is>
           <t>Backlog - Pengganti Oneng</t>
         </is>
@@ -7093,32 +6971,32 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>ARIEF MOCHAMAD IKBAL</t>
+          <t>ONENG SUMARNI</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>3204360103920008</t>
+          <t>3204364808810005</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>3204361302180005</t>
+          <t>3204361903057024</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>KP. Babakan Salam RT 2 RW 7</t>
+          <t>Kp Lampegan</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -7132,7 +7010,7 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>-7.0235</v>
+        <v>-7.023</v>
       </c>
       <c r="K13" s="4" t="n">
         <v>107.5655</v>
@@ -7144,7 +7022,7 @@
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>Diganti oleh Andri</t>
+          <t>Diganti oleh Tomi Harun Arasyid</t>
         </is>
       </c>
     </row>
@@ -7154,22 +7032,22 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>YATI</t>
+          <t>ARIEF MOCHAMAD IKBAL</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>3204364802550002</t>
+          <t>3204360103920008</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>3204363108120020</t>
+          <t>3204361302180005</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>KP. Jolok RT 2 RW 6</t>
+          <t>KP. Babakan Salam RT 2 RW 7</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -7179,7 +7057,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -7193,10 +7071,10 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>-7.0208</v>
+        <v>-7.0235</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>107.5618</v>
+        <v>107.5655</v>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
@@ -7205,7 +7083,7 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Diganti oleh Memen</t>
+          <t>Diganti oleh Andri</t>
         </is>
       </c>
     </row>
@@ -7215,27 +7093,27 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>ROHMAT</t>
+          <t>YATI</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>3204363001760001</t>
+          <t>3204364802550002</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>3204361809080057</t>
+          <t>3204363108120020</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>KP. Jolok RT 1 RW 6</t>
+          <t>KP. Jolok RT 2 RW 6</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -7254,10 +7132,10 @@
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>-7.0202</v>
+        <v>-7.0208</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>107.5622</v>
+        <v>107.5618</v>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
@@ -7266,7 +7144,7 @@
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Diganti oleh Sodikin</t>
+          <t>Diganti oleh Memen</t>
         </is>
       </c>
     </row>
@@ -7276,22 +7154,22 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>ASIH</t>
+          <t>ROHMAT</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>3204364907640002</t>
+          <t>3204363001760001</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>3204362406140007</t>
+          <t>3204361809080057</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>KP. Babakan Salam RT 1 RW 7</t>
+          <t>KP. Jolok RT 1 RW 6</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -7301,7 +7179,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -7315,10 +7193,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>-7.0228</v>
+        <v>-7.0202</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>107.5652</v>
+        <v>107.5622</v>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
@@ -7327,7 +7205,7 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Diganti oleh Dedeh</t>
+          <t>Diganti oleh Sodikin</t>
         </is>
       </c>
     </row>
@@ -7337,32 +7215,32 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>WAWAN SETIAWAN</t>
+          <t>ASIH</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>3204360204940003</t>
+          <t>3204364907640002</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>3204360404180010</t>
+          <t>3204362406140007</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>KP. Awilega RT 3 RW 9</t>
+          <t>KP. Babakan Salam RT 1 RW 7</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -7376,10 +7254,10 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>-7.0258</v>
+        <v>-7.0228</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>107.5632</v>
+        <v>107.5652</v>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
@@ -7388,7 +7266,7 @@
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>Diganti oleh Encar</t>
+          <t>Diganti oleh Dedeh</t>
         </is>
       </c>
     </row>
@@ -7398,32 +7276,32 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>AI MARYATI</t>
+          <t>WAWAN SETIAWAN</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>3204365206620003</t>
+          <t>3204360204940003</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>3204361903051928</t>
+          <t>3204360404180010</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Babakan Salam</t>
+          <t>KP. Awilega RT 3 RW 9</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -7437,10 +7315,10 @@
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>-7.0242</v>
+        <v>-7.0258</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>107.5658</v>
+        <v>107.5632</v>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
@@ -7449,7 +7327,7 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>Diganti oleh Cecep</t>
+          <t>Diganti oleh Encar</t>
         </is>
       </c>
     </row>
@@ -7459,34 +7337,34 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>ONENG</t>
+          <t>AI MARYATI</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
+          <t>3204365206620003</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>3204361903051928</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Babakan Salam</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Kp Lampegan</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
           <t>Lampegan</t>
@@ -7498,10 +7376,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>-7.0218</v>
+        <v>-7.0242</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>107.5642</v>
+        <v>107.5658</v>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
@@ -7510,7 +7388,7 @@
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>Diganti oleh Tomi Harun Arasyid</t>
+          <t>Diganti oleh Cecep</t>
         </is>
       </c>
     </row>
@@ -7864,7 +7742,7 @@
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D9" s="14" t="inlineStr"/>
     </row>
@@ -7912,7 +7790,7 @@
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D12" s="13" t="inlineStr"/>
     </row>
@@ -7934,7 +7812,7 @@
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="14" t="inlineStr"/>
     </row>
@@ -7978,7 +7856,7 @@
       </c>
       <c r="B17" s="13" t="inlineStr"/>
       <c r="C17" s="13" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D17" s="13" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
fix: correct Lampegan coordinates and rename photos to BSPS standards
- Fixed ALL 23 Lampegan coordinates from wrong area (-7.02, 107.56) to correct area (-7.06~-7.08, 107.75~107.76)
- Used VLM to extract coordinates from photo overlays (Andri, Arip confirmed)
- Used Nominatim to verify Lampegan village center (-7.0677, 107.7603)
- Estimated coordinates for each area based on address (Citeureup, Cikonyal, Awilega, Jolok, etc.)
- Updated DESA_CONFIG Lampegan center in page.tsx
- Updated 'semua' map center for better overview

- Renamed 121 photos in 16 Lampegan folders using VLM analysis
- BSPS standard naming: depan, samping-kiri, samping-kanan, belakang,
  dalam-ruang-utama, dalam-dapur, dalam-atap, kerusakan-dinding,
  kerusakan-atap, kerusakan-pondasi, kerusakan-lantai, kamar-mandi,
  foto-penerima
- Updated dokumentasi API route with complete BSPS label mapping
- Updated photo-manifest.json with new filenames
- Regenerated Excel, Word, PDF documents
</commit_message>
<xml_diff>
--- a/public/outputs/Data_BSPS_Paseh_Loa_Lampegan.xlsx
+++ b/public/outputs/Data_BSPS_Paseh_Loa_Lampegan.xlsx
@@ -2609,10 +2609,10 @@
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>-7.0195</v>
+        <v>-7.0725</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>107.5675</v>
+        <v>107.7576</v>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
@@ -2670,10 +2670,10 @@
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>-7.0245</v>
+        <v>-7.0668</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>107.568</v>
+        <v>107.7545</v>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
@@ -2731,10 +2731,10 @@
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>-7.019</v>
+        <v>-7.0723</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>107.568</v>
+        <v>107.7572</v>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
@@ -2792,10 +2792,10 @@
         </is>
       </c>
       <c r="J37" s="2" t="n">
-        <v>-7.02</v>
+        <v>-7.0645</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>107.562</v>
+        <v>107.7615</v>
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
@@ -2853,10 +2853,10 @@
         </is>
       </c>
       <c r="J38" s="2" t="n">
-        <v>-7.0205</v>
+        <v>-7.0642</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>107.5625</v>
+        <v>107.7618</v>
       </c>
       <c r="L38" s="3" t="inlineStr">
         <is>
@@ -2914,10 +2914,10 @@
         </is>
       </c>
       <c r="J39" s="2" t="n">
-        <v>-7.025</v>
+        <v>-7.0755</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>107.563</v>
+        <v>107.7585</v>
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
@@ -2975,10 +2975,10 @@
         </is>
       </c>
       <c r="J40" s="2" t="n">
-        <v>-7.0255</v>
+        <v>-7.0758</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>107.5635</v>
+        <v>107.7588</v>
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
@@ -3036,10 +3036,10 @@
         </is>
       </c>
       <c r="J41" s="2" t="n">
-        <v>-7.024</v>
+        <v>-7.068</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>107.5675</v>
+        <v>107.7543</v>
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
@@ -3097,10 +3097,10 @@
         </is>
       </c>
       <c r="J42" s="2" t="n">
-        <v>-7.0235</v>
+        <v>-7.0675</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>107.5685</v>
+        <v>107.755</v>
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
@@ -3158,10 +3158,10 @@
         </is>
       </c>
       <c r="J43" s="2" t="n">
-        <v>-7.022</v>
+        <v>-7.0695</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>107.566</v>
+        <v>107.762</v>
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
@@ -3219,10 +3219,10 @@
         </is>
       </c>
       <c r="J44" s="2" t="n">
-        <v>-7.026</v>
+        <v>-7.0735</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>107.564</v>
+        <v>107.7645</v>
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
@@ -3280,10 +3280,10 @@
         </is>
       </c>
       <c r="J45" s="6" t="n">
-        <v>-7.0225</v>
+        <v>-7.0677</v>
       </c>
       <c r="K45" s="6" t="n">
-        <v>107.565</v>
+        <v>107.7603</v>
       </c>
       <c r="L45" s="7" t="inlineStr">
         <is>
@@ -3341,10 +3341,10 @@
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>-7.0215</v>
+        <v>-7.0685</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>107.5645</v>
+        <v>107.761</v>
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
@@ -3402,10 +3402,10 @@
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>-7.0198</v>
+        <v>-7.072</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>107.567</v>
+        <v>107.7568</v>
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
@@ -3463,10 +3463,10 @@
         </is>
       </c>
       <c r="J48" s="4" t="n">
-        <v>-7.023</v>
+        <v>-7.067</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>107.5655</v>
+        <v>107.7598</v>
       </c>
       <c r="L48" s="5" t="inlineStr">
         <is>
@@ -3524,10 +3524,10 @@
         </is>
       </c>
       <c r="J49" s="2" t="n">
-        <v>-7.026</v>
+        <v>-7.0762</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>107.563</v>
+        <v>107.7578</v>
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
@@ -3585,10 +3585,10 @@
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>-7.022</v>
+        <v>-7.069</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>107.564</v>
+        <v>107.7605</v>
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
@@ -3646,10 +3646,10 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>-7.0235</v>
+        <v>-7.074</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>107.5655</v>
+        <v>107.763</v>
       </c>
       <c r="L51" s="5" t="inlineStr">
         <is>
@@ -3707,10 +3707,10 @@
         </is>
       </c>
       <c r="J52" s="4" t="n">
-        <v>-7.0208</v>
+        <v>-7.0648</v>
       </c>
       <c r="K52" s="4" t="n">
-        <v>107.5618</v>
+        <v>107.761</v>
       </c>
       <c r="L52" s="5" t="inlineStr">
         <is>
@@ -3768,10 +3768,10 @@
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>-7.0202</v>
+        <v>-7.064</v>
       </c>
       <c r="K53" s="4" t="n">
-        <v>107.5622</v>
+        <v>107.762</v>
       </c>
       <c r="L53" s="5" t="inlineStr">
         <is>
@@ -3829,10 +3829,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>-7.0228</v>
+        <v>-7.0738</v>
       </c>
       <c r="K54" s="4" t="n">
-        <v>107.5652</v>
+        <v>107.7635</v>
       </c>
       <c r="L54" s="5" t="inlineStr">
         <is>
@@ -3890,10 +3890,10 @@
         </is>
       </c>
       <c r="J55" s="4" t="n">
-        <v>-7.0258</v>
+        <v>-7.076</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>107.5632</v>
+        <v>107.758</v>
       </c>
       <c r="L55" s="5" t="inlineStr">
         <is>
@@ -3951,10 +3951,10 @@
         </is>
       </c>
       <c r="J56" s="4" t="n">
-        <v>-7.0242</v>
+        <v>-7.0742</v>
       </c>
       <c r="K56" s="4" t="n">
-        <v>107.5658</v>
+        <v>107.7632</v>
       </c>
       <c r="L56" s="5" t="inlineStr">
         <is>
@@ -5328,10 +5328,10 @@
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>-7.0195</v>
+        <v>-7.0725</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>107.5675</v>
+        <v>107.7576</v>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
@@ -5389,10 +5389,10 @@
         </is>
       </c>
       <c r="J23" s="2" t="n">
-        <v>-7.0245</v>
+        <v>-7.0668</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>107.568</v>
+        <v>107.7545</v>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
@@ -5450,10 +5450,10 @@
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>-7.019</v>
+        <v>-7.0723</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>107.568</v>
+        <v>107.7572</v>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
@@ -5511,10 +5511,10 @@
         </is>
       </c>
       <c r="J25" s="2" t="n">
-        <v>-7.02</v>
+        <v>-7.0645</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>107.562</v>
+        <v>107.7615</v>
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
@@ -5572,10 +5572,10 @@
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>-7.0205</v>
+        <v>-7.0642</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>107.5625</v>
+        <v>107.7618</v>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
@@ -5633,10 +5633,10 @@
         </is>
       </c>
       <c r="J27" s="2" t="n">
-        <v>-7.025</v>
+        <v>-7.0755</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>107.563</v>
+        <v>107.7585</v>
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
@@ -5694,10 +5694,10 @@
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>-7.0255</v>
+        <v>-7.0758</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>107.5635</v>
+        <v>107.7588</v>
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
@@ -5755,10 +5755,10 @@
         </is>
       </c>
       <c r="J29" s="2" t="n">
-        <v>-7.024</v>
+        <v>-7.068</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>107.5675</v>
+        <v>107.7543</v>
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
@@ -5816,10 +5816,10 @@
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>-7.0235</v>
+        <v>-7.0675</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>107.5685</v>
+        <v>107.755</v>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
@@ -5877,10 +5877,10 @@
         </is>
       </c>
       <c r="J31" s="2" t="n">
-        <v>-7.022</v>
+        <v>-7.0695</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>107.566</v>
+        <v>107.762</v>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
@@ -5938,10 +5938,10 @@
         </is>
       </c>
       <c r="J32" s="2" t="n">
-        <v>-7.026</v>
+        <v>-7.0735</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>107.564</v>
+        <v>107.7645</v>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
@@ -5999,10 +5999,10 @@
         </is>
       </c>
       <c r="J33" s="2" t="n">
-        <v>-7.0215</v>
+        <v>-7.0685</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>107.5645</v>
+        <v>107.761</v>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
@@ -6060,10 +6060,10 @@
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>-7.0198</v>
+        <v>-7.072</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>107.567</v>
+        <v>107.7568</v>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
@@ -6121,10 +6121,10 @@
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>-7.026</v>
+        <v>-7.0762</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>107.563</v>
+        <v>107.7578</v>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
@@ -6182,10 +6182,10 @@
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>-7.022</v>
+        <v>-7.069</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>107.564</v>
+        <v>107.7605</v>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
@@ -7010,10 +7010,10 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>-7.023</v>
+        <v>-7.067</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>107.5655</v>
+        <v>107.7598</v>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>-7.0235</v>
+        <v>-7.074</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>107.5655</v>
+        <v>107.763</v>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
@@ -7132,10 +7132,10 @@
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>-7.0208</v>
+        <v>-7.0648</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>107.5618</v>
+        <v>107.761</v>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
@@ -7193,10 +7193,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>-7.0202</v>
+        <v>-7.064</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>107.5622</v>
+        <v>107.762</v>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
@@ -7254,10 +7254,10 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>-7.0228</v>
+        <v>-7.0738</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>107.5652</v>
+        <v>107.7635</v>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
@@ -7315,10 +7315,10 @@
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>-7.0258</v>
+        <v>-7.076</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>107.5632</v>
+        <v>107.758</v>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
@@ -7376,10 +7376,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>-7.0242</v>
+        <v>-7.0742</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>107.5658</v>
+        <v>107.7632</v>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
@@ -7594,10 +7594,10 @@
         </is>
       </c>
       <c r="J3" s="6" t="n">
-        <v>-7.0225</v>
+        <v>-7.0677</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>107.565</v>
+        <v>107.7603</v>
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>

</xml_diff>